<commit_message>
Added excel doc for ICP Instrument,Feedbackform ,InstrumentPrice list
</commit_message>
<xml_diff>
--- a/src/assets/CifDocumentsTemplates/100005.xlsx
+++ b/src/assets/CifDocumentsTemplates/100005.xlsx
@@ -11,17 +11,168 @@
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_GoBack" localSheetId="0">Sheet1!$B$8</definedName>
+  </definedNames>
   <calcPr calcId="125725"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
+  <si>
+    <t>Instrument Name</t>
+  </si>
+  <si>
+    <t>Internal (per sample)</t>
+  </si>
+  <si>
+    <t>Academia/R&amp;D (per sample)</t>
+  </si>
+  <si>
+    <t>Industry (per sample)</t>
+  </si>
+  <si>
+    <t>Inductively Coupled Plasma Optical Emission Spectrometry (PerkinElmer ICP-OES Optima 8000)</t>
+  </si>
+  <si>
+    <r>
+      <t>500/- per sample (upto 1 elements)</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>**</t>
+    </r>
+  </si>
+  <si>
+    <t>and</t>
+  </si>
+  <si>
+    <t>+ 150/- extra for additional element</t>
+  </si>
+  <si>
+    <r>
+      <t>Note:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> [1] Standards will be provided by the user only. [2] 750/- per sample will be charged extra for sample preparation (i.e., acid digestion).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>**</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>850/- per sample (upto 1 elements)</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>**</t>
+    </r>
+  </si>
+  <si>
+    <t>+ 175/- extra for additional element</t>
+  </si>
+  <si>
+    <r>
+      <t>**</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>1500/- per sample (upto 1 elements)</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> **</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> + 200/- extra for additional element</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">+ 200/- extra for additional element </t>
+  </si>
+  <si>
+    <r>
+      <t>Note:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> [1] Standards will be provided by the user only. [2] 1000/- per sample will be charged extra for sample preparation (i.e., acid digestion).</t>
+    </r>
+  </si>
+  <si>
+    <t>Central instrumentation FACILITY (CIF)</t>
+  </si>
+  <si>
+    <t>Lovely Professional University</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jalandhar - Delhi G.T. Road, Phagwara, Punjab (India) - 144411, </t>
+  </si>
+  <si>
+    <t>Telephone no: +911824444535, Fax no: +91824-506111, Email-id: cif@lpu.co.in</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -37,6 +188,43 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -46,7 +234,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -55,64 +243,128 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <left style="medium">
         <color indexed="64"/>
       </left>
-      <right style="thin">
+      <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin">
+      <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
-      <right/>
-      <top style="thin">
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
         <color indexed="64"/>
       </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
       <left/>
-      <right/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
       <top/>
-      <bottom style="thin">
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -408,187 +660,115 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J14"/>
+  <dimension ref="B2:E12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="11" width="21.28515625" customWidth="1"/>
+    <col min="2" max="2" width="25.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="70.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="11" width="21.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
-      <c r="A1" s="5"/>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="6"/>
-    </row>
-    <row r="2" spans="1:10">
-      <c r="A2" s="3"/>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-    </row>
-    <row r="3" spans="1:10">
-      <c r="A3" s="2"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-    </row>
-    <row r="4" spans="1:10">
-      <c r="A4" s="2"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-    </row>
-    <row r="5" spans="1:10">
-      <c r="A5" s="2"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
-    </row>
-    <row r="6" spans="1:10">
-      <c r="A6" s="2"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-    </row>
-    <row r="7" spans="1:10">
-      <c r="A7" s="2"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
-    </row>
-    <row r="8" spans="1:10">
-      <c r="A8" s="2"/>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-      <c r="J8" s="1"/>
-    </row>
-    <row r="9" spans="1:10">
-      <c r="A9" s="2"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
-      <c r="J9" s="1"/>
-    </row>
-    <row r="10" spans="1:10">
-      <c r="A10" s="2"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1"/>
-      <c r="J10" s="1"/>
-    </row>
-    <row r="11" spans="1:10">
-      <c r="A11" s="2"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
-      <c r="J11" s="1"/>
-    </row>
-    <row r="12" spans="1:10">
-      <c r="A12" s="2"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-      <c r="G12" s="1"/>
-      <c r="H12" s="1"/>
-      <c r="I12" s="1"/>
-      <c r="J12" s="1"/>
-    </row>
-    <row r="13" spans="1:10">
-      <c r="A13" s="2"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1"/>
-      <c r="J13" s="1"/>
-    </row>
-    <row r="14" spans="1:10">
-      <c r="A14" s="7"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7"/>
-      <c r="H14" s="7"/>
-      <c r="I14" s="7"/>
-      <c r="J14" s="7"/>
+    <row r="2" spans="2:5" ht="15.75">
+      <c r="C2" s="10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5" ht="15.75">
+      <c r="C3" s="10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5">
+      <c r="C4" s="11" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5">
+      <c r="C5" s="11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" ht="15.75" thickBot="1">
+      <c r="C6" s="11"/>
+    </row>
+    <row r="7" spans="2:5" ht="48" thickBot="1">
+      <c r="B7" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" ht="60.75">
+      <c r="B8" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5">
+      <c r="B9" s="7"/>
+      <c r="C9" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" ht="30">
+      <c r="B10" s="7"/>
+      <c r="C10" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" ht="105">
+      <c r="B11" s="7"/>
+      <c r="C11" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" ht="15.75" thickBot="1">
+      <c r="B12" s="9"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:J1"/>
-    <mergeCell ref="A14:J14"/>
+  <mergeCells count="1">
+    <mergeCell ref="B8:B12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>